<commit_message>
Repair the HPfinance sheet's broken monthly-payment formula
Every hire purchase agreement row after the first one in each block
charged #REF!/H<r> for its monthly payment instead of the working
formula the first row carries: (E+F+G)/H, amount financed plus admin
charges plus total interest, over the term in months.

Rewrote every occurrence of IF(H<r>>0,#REF!/H<r>," ") to
IF(E<r>>0,(E<r>+F<r>+G<r>)/H<r>," "), the same shape row 8 (SE, Ltd)
and row 22 (SE) / row 34 (Ltd) already use. 6 rows in SE, 18 in Ltd.
No #REF! remains on either sheet afterwards. J and K on these rows
were already correct and untouched.

A new test reads both templates' HPfinance sheets directly via JSZip
(no LibreOffice needed) and asserts every repaired row's I/J/K
formulas have the same shape as their block's working master, after
normalising away the row number.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Fixedassets.xlsx
+++ b/app/templates/ltd/Fixedassets.xlsx
@@ -8648,7 +8648,7 @@
       <c r="G10" s="83"/>
       <c r="H10" s="89"/>
       <c r="I10" s="81" t="str">
-        <f>IF(H10&gt;0,#REF!/H10," ")</f>
+        <f>IF(E10&gt;0,(E10+F10+G10)/H10," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J10" s="81" t="str">
@@ -8687,7 +8687,7 @@
       <c r="G12" s="83"/>
       <c r="H12" s="89"/>
       <c r="I12" s="81" t="str">
-        <f>IF(H12&gt;0,#REF!/H12," ")</f>
+        <f>IF(E12&gt;0,(E12+F12+G12)/H12," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J12" s="81" t="str">
@@ -8726,7 +8726,7 @@
       <c r="G14" s="83"/>
       <c r="H14" s="89"/>
       <c r="I14" s="81" t="str">
-        <f>IF(H14&gt;0,#REF!/H14," ")</f>
+        <f>IF(E14&gt;0,(E14+F14+G14)/H14," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J14" s="81" t="str">
@@ -8765,7 +8765,7 @@
       <c r="G16" s="83"/>
       <c r="H16" s="89"/>
       <c r="I16" s="81" t="str">
-        <f>IF(H16&gt;0,#REF!/H16," ")</f>
+        <f>IF(E16&gt;0,(E16+F16+G16)/H16," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J16" s="81" t="str">
@@ -8804,7 +8804,7 @@
       <c r="G18" s="83"/>
       <c r="H18" s="89"/>
       <c r="I18" s="81" t="str">
-        <f>IF(H18&gt;0,#REF!/H18," ")</f>
+        <f>IF(E18&gt;0,(E18+F18+G18)/H18," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J18" s="81" t="str">
@@ -8843,7 +8843,7 @@
       <c r="G20" s="83"/>
       <c r="H20" s="89"/>
       <c r="I20" s="81" t="str">
-        <f>IF(H20&gt;0,#REF!/H20," ")</f>
+        <f>IF(E20&gt;0,(E20+F20+G20)/H20," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J20" s="81" t="str">
@@ -8882,7 +8882,7 @@
       <c r="G22" s="83"/>
       <c r="H22" s="89"/>
       <c r="I22" s="81" t="str">
-        <f>IF(H22&gt;0,#REF!/H22," ")</f>
+        <f>IF(E22&gt;0,(E22+F22+G22)/H22," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J22" s="81" t="str">
@@ -8921,7 +8921,7 @@
       <c r="G24" s="83"/>
       <c r="H24" s="89"/>
       <c r="I24" s="81" t="str">
-        <f>IF(H24&gt;0,#REF!/H24," ")</f>
+        <f>IF(E24&gt;0,(E24+F24+G24)/H24," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J24" s="81" t="str">
@@ -8960,7 +8960,7 @@
       <c r="G26" s="83"/>
       <c r="H26" s="89"/>
       <c r="I26" s="81" t="str">
-        <f>IF(H26&gt;0,#REF!/H26," ")</f>
+        <f>IF(E26&gt;0,(E26+F26+G26)/H26," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J26" s="81" t="str">
@@ -9156,7 +9156,7 @@
       <c r="G36" s="83"/>
       <c r="H36" s="89"/>
       <c r="I36" s="81" t="str">
-        <f>IF(H36&gt;0,#REF!/H36," ")</f>
+        <f>IF(E36&gt;0,(E36+F36+G36)/H36," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J36" s="81" t="str">
@@ -9195,7 +9195,7 @@
       <c r="G38" s="83"/>
       <c r="H38" s="89"/>
       <c r="I38" s="81" t="str">
-        <f>IF(H38&gt;0,#REF!/H38," ")</f>
+        <f>IF(E38&gt;0,(E38+F38+G38)/H38," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J38" s="81" t="str">
@@ -9234,7 +9234,7 @@
       <c r="G40" s="83"/>
       <c r="H40" s="89"/>
       <c r="I40" s="81" t="str">
-        <f>IF(H40&gt;0,#REF!/H40," ")</f>
+        <f>IF(E40&gt;0,(E40+F40+G40)/H40," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J40" s="81" t="str">
@@ -9273,7 +9273,7 @@
       <c r="G42" s="83"/>
       <c r="H42" s="89"/>
       <c r="I42" s="81" t="str">
-        <f>IF(H42&gt;0,#REF!/H42," ")</f>
+        <f>IF(E42&gt;0,(E42+F42+G42)/H42," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J42" s="81" t="str">
@@ -9312,7 +9312,7 @@
       <c r="G44" s="83"/>
       <c r="H44" s="89"/>
       <c r="I44" s="81" t="str">
-        <f>IF(H44&gt;0,#REF!/H44," ")</f>
+        <f>IF(E44&gt;0,(E44+F44+G44)/H44," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J44" s="81" t="str">
@@ -9351,7 +9351,7 @@
       <c r="G46" s="83"/>
       <c r="H46" s="89"/>
       <c r="I46" s="81" t="str">
-        <f>IF(H46&gt;0,#REF!/H46," ")</f>
+        <f>IF(E46&gt;0,(E46+F46+G46)/H46," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J46" s="81" t="str">
@@ -9390,7 +9390,7 @@
       <c r="G48" s="83"/>
       <c r="H48" s="89"/>
       <c r="I48" s="81" t="str">
-        <f>IF(H48&gt;0,#REF!/H48," ")</f>
+        <f>IF(E48&gt;0,(E48+F48+G48)/H48," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J48" s="81" t="str">
@@ -9429,7 +9429,7 @@
       <c r="G50" s="83"/>
       <c r="H50" s="89"/>
       <c r="I50" s="81" t="str">
-        <f>IF(H50&gt;0,#REF!/H50," ")</f>
+        <f>IF(E50&gt;0,(E50+F50+G50)/H50," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J50" s="81" t="str">
@@ -9468,7 +9468,7 @@
       <c r="G52" s="83"/>
       <c r="H52" s="89"/>
       <c r="I52" s="81" t="str">
-        <f>IF(H52&gt;0,#REF!/H52," ")</f>
+        <f>IF(E52&gt;0,(E52+F52+G52)/H52," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="J52" s="81" t="str">

</xml_diff>